<commit_message>
Remove measurement group validation
</commit_message>
<xml_diff>
--- a/inst/templates/english/data/template.xlsx
+++ b/inst/templates/english/data/template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\dirt-data-reports\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\inst\templates\english\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6505725E-5C9D-4713-BDD8-EBA7FCE1F7AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDEEA1DA-2A46-482D-8723-B875BDD8A520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="466">
   <si>
     <t>year</t>
   </si>
@@ -2111,53 +2111,6 @@
     <t>Use the Data Dictionary to control how measurements appear in the Project Results section of the report.</t>
   </si>
   <si>
-    <t>◦ Only the following values are currently supported. Custom groups are not allowed and will fail validation.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">▪ </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>English</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Physical, Biological, Chemical, Plant Essential Macro Nutrients, Plant Essential Micro Nutrients</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">▪ </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Spanish</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>: Mediciones físicas, Mediciones biológicas, Mediciones químicas, Macronutrientes esenciales para plantas, Micronutrientes esenciales para plantas</t>
-    </r>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">• </t>
     </r>
@@ -2629,7 +2582,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2653,12 +2606,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2961,7 +2908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E845E3A-25D1-4A93-81A5-4976079DA411}">
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="182.88671875" style="4" customWidth="1"/>
@@ -3008,7 +2955,7 @@
     </row>
     <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
@@ -3048,7 +2995,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
@@ -3108,12 +3055,12 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
@@ -3153,7 +3100,7 @@
     </row>
     <row r="42" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
@@ -3168,42 +3115,27 @@
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="10" t="s">
         <v>464</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="10" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="11" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="11" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="6" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="6" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
-        <v>467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>